<commit_message>
Release DocRedock v0.1.1 public beta
</commit_message>
<xml_diff>
--- a/outputs/japanese-system-design-ocr-check/japanese-system-design-ocr-sample.xlsx
+++ b/outputs/japanese-system-design-ocr-check/japanese-system-design-ocr-sample.xlsx
@@ -8,6 +8,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCR期待値" sheetId="4" r:id="R6225bb067055406e"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="画面設計" sheetId="5" r:id="R9ac3b9e2340544b3"/>
   </x:sheets>
+  <calcPr xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
 </file>
 
@@ -1312,8 +1313,10 @@
       <x:c r="N2" s="6"/>
     </x:row>
     <x:row r="3" ht="16.5" customHeight="1">
-      <x:c r="A3" s="9" t="str">
-        <x:v>Excel方眼紙・シーケンス・業務フロー・貼付画面・OCRを含むRTMD変換確認用サンプル</x:v>
+      <x:c r="A3" s="9" t="inlineStr">
+        <is xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <t>Excel方眼紙・シーケンス・業務フロー・貼付画面・OCRを含むDRMD変換確認用サンプル</t>
+        </is>
       </x:c>
       <x:c r="B3" s="9"/>
       <x:c r="C3" s="9"/>
@@ -1434,8 +1437,10 @@
         <x:v>金額(円)</x:v>
       </x:c>
       <x:c r="H8" s="3"/>
-      <x:c r="I8" s="35" t="str">
-        <x:v>RTMD確認ポイント</x:v>
+      <x:c r="I8" s="35" t="inlineStr">
+        <is xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <t>DRMD確認ポイント</t>
+        </is>
       </x:c>
       <x:c r="J8" s="35"/>
       <x:c r="K8" s="35"/>
@@ -1651,8 +1656,10 @@
       <x:c r="N15" s="3"/>
     </x:row>
     <x:row r="16" ht="16.5" customHeight="1">
-      <x:c r="A16" s="53" t="str">
-        <x:v>凡例：青字＝入力値／緑字＝数式。RTMDのMarkdownでは数式セルを `=式` → 計算結果 の形式で投影し、計算結果側は参照専用です。</x:v>
+      <x:c r="A16" s="53" t="inlineStr">
+        <is xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <t>凡例：青字＝入力値／緑字＝数式。DRMDのMarkdownでは数式セルを `=式` → 計算結果 の形式で投影し、計算結果側は参照専用です。</t>
+        </is>
       </x:c>
       <x:c r="B16" s="54"/>
       <x:c r="C16" s="54"/>
@@ -4446,8 +4453,10 @@
       <x:c r="Z2" s="6"/>
     </x:row>
     <x:row r="3" ht="15" customHeight="1">
-      <x:c r="A3" s="9" t="str">
-        <x:v>Excelセル方眼紙の上に画面キャプチャを貼り付けた実務風レイアウト。貼付画像はRTMDのアセット抽出・OCR対象</x:v>
+      <x:c r="A3" s="9" t="inlineStr">
+        <is xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <t>Excelセル方眼紙の上に画面キャプチャを貼り付けた実務風レイアウト。貼付画像はDRMDのアセット抽出・OCR対象</t>
+        </is>
       </x:c>
       <x:c r="B3" s="9"/>
       <x:c r="C3" s="9"/>

</xml_diff>